<commit_message>
Update sector analysis (VDS_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/sector analysis (VDS_s) 0.xlsx
+++ b/clustering/sepsectors/sector analysis (VDS_s) 0.xlsx
@@ -5,27 +5,27 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\.spyder-py3\ITMO-3\clustering\sepsectors\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Пром. производство" sheetId="3" r:id="rId1"/>
-    <sheet name="Сельхоз" sheetId="1" r:id="rId2"/>
-    <sheet name="Административный" sheetId="2" r:id="rId3"/>
-    <sheet name="Логистика" sheetId="4" r:id="rId4"/>
-    <sheet name="Добыча" sheetId="5" r:id="rId5"/>
-    <sheet name="Торговля" sheetId="6" r:id="rId6"/>
-    <sheet name="Наука" sheetId="7" r:id="rId7"/>
+    <sheet name="Логистика" sheetId="4" r:id="rId2"/>
+    <sheet name="Наука" sheetId="7" r:id="rId3"/>
+    <sheet name="Торговля" sheetId="6" r:id="rId4"/>
+    <sheet name="Сельхоз" sheetId="1" r:id="rId5"/>
+    <sheet name="Административный" sheetId="2" r:id="rId6"/>
+    <sheet name="Добыча" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="93">
   <si>
     <t>sector</t>
   </si>
@@ -395,7 +395,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -408,9 +408,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1454,13 +1451,13 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="8">
+      <c r="C32" s="7">
         <v>2023</v>
       </c>
       <c r="D32" s="3">
@@ -2167,7 +2164,7 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B64" s="6" t="s">
+      <c r="B64" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D64" s="3">
@@ -2176,10 +2173,10 @@
       </c>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B65" s="7"/>
+      <c r="B65" s="6"/>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B66" s="7" t="s">
+      <c r="B66" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D66" s="3">
@@ -2200,7 +2197,7 @@
       </c>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B67" s="7" t="s">
+      <c r="B67" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D67" s="3">
@@ -2221,7 +2218,7 @@
       </c>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C69" s="7" t="s">
+      <c r="C69" s="6" t="s">
         <v>52</v>
       </c>
       <c r="D69" s="3">
@@ -2344,825 +2341,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="97.85546875" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D2" s="3">
-        <v>3292837.3871137551</v>
-      </c>
-      <c r="E2" s="3">
-        <v>5258.5701260400001</v>
-      </c>
-      <c r="F2" s="4">
-        <v>1.0604360748915839E-2</v>
-      </c>
-      <c r="G2" s="4">
-        <v>1.868819729404374E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D3" s="3">
-        <v>3097084.3107878752</v>
-      </c>
-      <c r="E3" s="3">
-        <v>4162.4721680000002</v>
-      </c>
-      <c r="F3" s="4">
-        <v>1.4081114307645259E-3</v>
-      </c>
-      <c r="G3" s="4">
-        <v>3.9573959548935052E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D4" s="3">
-        <v>2652658.7944572391</v>
-      </c>
-      <c r="E4" s="3">
-        <v>4253.6615775199998</v>
-      </c>
-      <c r="F4" s="4">
-        <v>2.8806641846538372E-3</v>
-      </c>
-      <c r="G4" s="4">
-        <v>1.8380008135386839E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D5" s="3">
-        <v>2480166.278394436</v>
-      </c>
-      <c r="E5" s="3">
-        <v>4510.0316159999993</v>
-      </c>
-      <c r="F5" s="4">
-        <v>1.003512255644462E-3</v>
-      </c>
-      <c r="G5" s="4">
-        <v>1.2206708220113729E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D6" s="3">
-        <v>331647.0310656284</v>
-      </c>
-      <c r="E6" s="3">
-        <v>964.84556195999994</v>
-      </c>
-      <c r="F6" s="4">
-        <v>7.4163848413873461E-4</v>
-      </c>
-      <c r="G6" s="4">
-        <v>3.6380912535570372E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D7" s="3">
-        <v>255261.79722573471</v>
-      </c>
-      <c r="E7" s="3">
-        <v>888.20773440000005</v>
-      </c>
-      <c r="F7" s="4">
-        <v>1.2066660967819649E-3</v>
-      </c>
-      <c r="G7" s="4">
-        <v>2.863735386990569E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D8" s="3">
-        <v>238996.75153477999</v>
-      </c>
-      <c r="E8" s="3">
-        <v>863.40619829999991</v>
-      </c>
-      <c r="F8" s="4">
-        <v>7.0023981897559661E-4</v>
-      </c>
-      <c r="G8" s="4">
-        <v>9.1753228267274999E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D9" s="3">
-        <v>218314.63160777459</v>
-      </c>
-      <c r="E9" s="3">
-        <v>897.65553599999998</v>
-      </c>
-      <c r="F9" s="4">
-        <v>4.6312642581418888E-4</v>
-      </c>
-      <c r="G9" s="4">
-        <v>5.3328786021100191E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D10" s="3">
-        <v>177476.11420904889</v>
-      </c>
-      <c r="E10" s="3">
-        <v>1454.99992092</v>
-      </c>
-      <c r="F10" s="4">
-        <v>2.7347370558508639E-4</v>
-      </c>
-      <c r="G10" s="4">
-        <v>8.7625687236728058E-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D11" s="3">
-        <v>149725.9222474432</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1319.2765561000001</v>
-      </c>
-      <c r="F11" s="4">
-        <v>9.5143491498901212E-3</v>
-      </c>
-      <c r="G11" s="4">
-        <v>8.6555389370039323E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D12" s="3">
-        <v>123407.0292947656</v>
-      </c>
-      <c r="E12" s="3">
-        <v>769.72569599999997</v>
-      </c>
-      <c r="F12" s="4">
-        <v>1.643806367093142E-3</v>
-      </c>
-      <c r="G12" s="4">
-        <v>4.963035559098705E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D13" s="3">
-        <v>118648.02708896549</v>
-      </c>
-      <c r="E13" s="3">
-        <v>640.62859736000007</v>
-      </c>
-      <c r="F13" s="4">
-        <v>4.2703506076277667E-2</v>
-      </c>
-      <c r="G13" s="4">
-        <v>7.645975624855611E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="3">
-        <f>MEDIAN(D2:D13)</f>
-        <v>247129.27438025735</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B16" s="7"/>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="3">
-        <f>AVERAGE(D2:D7)</f>
-        <v>2018275.9331741116</v>
-      </c>
-      <c r="E17" s="3">
-        <f t="shared" ref="E17:G17" si="0">AVERAGE(E2:E7)</f>
-        <v>3339.6314639866664</v>
-      </c>
-      <c r="F17" s="4">
-        <f t="shared" si="0"/>
-        <v>2.974158866816561E-3</v>
-      </c>
-      <c r="G17" s="4">
-        <f t="shared" si="0"/>
-        <v>2.0187386386990346E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="3">
-        <f>AVERAGE(D8:D13)</f>
-        <v>171094.74599712962</v>
-      </c>
-      <c r="E18" s="3">
-        <f t="shared" ref="E18:G18" si="1">AVERAGE(E8:E13)</f>
-        <v>990.94875077999995</v>
-      </c>
-      <c r="F18" s="4">
-        <f t="shared" si="1"/>
-        <v>9.2164169239392999E-3</v>
-      </c>
-      <c r="G18" s="4">
-        <f t="shared" si="1"/>
-        <v>3.4335388058007936E-3</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState ref="A2:G13">
-    <sortCondition descending="1" ref="D2:D13"/>
-  </sortState>
-  <conditionalFormatting sqref="D2:D13">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E13">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F13">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G13">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17:D18">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E18">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F17:F18">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G18">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="73" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D2" s="3">
-        <v>971947.1589226143</v>
-      </c>
-      <c r="E2" s="3">
-        <v>21731.663739110001</v>
-      </c>
-      <c r="F2" s="4">
-        <v>3.0282081846115981E-5</v>
-      </c>
-      <c r="G2" s="4">
-        <v>5.0206173563068553E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D3" s="3">
-        <v>950234.48563991196</v>
-      </c>
-      <c r="E3" s="3">
-        <v>3253.0570836699999</v>
-      </c>
-      <c r="F3" s="4">
-        <v>3.2666995157709352E-4</v>
-      </c>
-      <c r="G3" s="4">
-        <v>1.167450820049999E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D4" s="3">
-        <v>840420.70663642394</v>
-      </c>
-      <c r="E4" s="3">
-        <v>22097.462448999999</v>
-      </c>
-      <c r="F4" s="4">
-        <v>1.047846559460851E-5</v>
-      </c>
-      <c r="G4" s="4">
-        <v>8.9257472528899238E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D5" s="3">
-        <v>130071.2900498806</v>
-      </c>
-      <c r="E5" s="3">
-        <v>866.32844524999996</v>
-      </c>
-      <c r="F5" s="4">
-        <v>1.8830176464184379E-3</v>
-      </c>
-      <c r="G5" s="4">
-        <v>2.5735129813919731E-4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D6" s="3">
-        <v>118956.3612196709</v>
-      </c>
-      <c r="E6" s="3">
-        <v>1090.8420791399999</v>
-      </c>
-      <c r="F6" s="4">
-        <v>6.857037460360029E-4</v>
-      </c>
-      <c r="G6" s="4">
-        <v>4.8025762850386331E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D7" s="3">
-        <v>106346.7598437235</v>
-      </c>
-      <c r="E7" s="3">
-        <v>1736.36278023</v>
-      </c>
-      <c r="F7" s="4">
-        <v>2.7534118528886658E-3</v>
-      </c>
-      <c r="G7" s="4">
-        <v>9.5257384161442811E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D8" s="3">
-        <v>85809.083743767143</v>
-      </c>
-      <c r="E8" s="3">
-        <v>2740.6294030899999</v>
-      </c>
-      <c r="F8" s="4">
-        <v>3.444045779906578E-2</v>
-      </c>
-      <c r="G8" s="4">
-        <v>2.7573625574766692E-4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="3">
-        <f>MEDIAN(D2:D8)</f>
-        <v>130071.2900498806</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="3">
-        <f>AVERAGE(D2:D4)</f>
-        <v>920867.45039964991</v>
-      </c>
-      <c r="E12" s="3">
-        <f t="shared" ref="E12:G12" si="0">AVERAGE(E2:E4)</f>
-        <v>15694.061090593334</v>
-      </c>
-      <c r="F12" s="4">
-        <f t="shared" si="0"/>
-        <v>1.2247683300593934E-4</v>
-      </c>
-      <c r="G12" s="4">
-        <f t="shared" si="0"/>
-        <v>5.0379384764155924E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="3">
-        <f>AVERAGE(D6:D8)</f>
-        <v>103704.06826905387</v>
-      </c>
-      <c r="E13" s="3">
-        <f t="shared" ref="E13:G13" si="1">AVERAGE(E6:E8)</f>
-        <v>1855.9447541533334</v>
-      </c>
-      <c r="F13" s="4">
-        <f t="shared" si="1"/>
-        <v>1.2626524465996816E-2</v>
-      </c>
-      <c r="G13" s="4">
-        <f t="shared" si="1"/>
-        <v>3.4272441001319369E-3</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="D2:D8">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E8">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F8">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G8">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D12:D13">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E12:E13">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F13">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G12:G13">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3474,7 +2652,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="3">
@@ -3483,7 +2661,7 @@
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="3">
@@ -3504,7 +2682,7 @@
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="3">
@@ -3525,7 +2703,7 @@
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>52</v>
       </c>
       <c r="D20" s="3">
@@ -3631,6 +2809,1207 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G17:G18">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="120.28515625" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2312764.5271400302</v>
+      </c>
+      <c r="E2" s="3">
+        <v>35420.059524999997</v>
+      </c>
+      <c r="F2" s="10">
+        <v>5.6205038026400662E-3</v>
+      </c>
+      <c r="G2" s="10">
+        <v>1.8864917830766969E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2056038.0691327541</v>
+      </c>
+      <c r="E3" s="3">
+        <v>35306.169047820003</v>
+      </c>
+      <c r="F3" s="10">
+        <v>7.4585983781851224E-3</v>
+      </c>
+      <c r="G3" s="10">
+        <v>1.5495337612500891E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1713109.9518803279</v>
+      </c>
+      <c r="E4" s="3">
+        <v>77023.192478700003</v>
+      </c>
+      <c r="F4" s="10">
+        <v>9.4864560705148846E-3</v>
+      </c>
+      <c r="G4" s="10">
+        <v>3.0572532777723999E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1230284.2821290109</v>
+      </c>
+      <c r="E5" s="3">
+        <v>94580.340012330009</v>
+      </c>
+      <c r="F5" s="10">
+        <v>4.1181927359240046E-3</v>
+      </c>
+      <c r="G5" s="10">
+        <v>2.9431664964802489E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1177149.00870383</v>
+      </c>
+      <c r="E6" s="3">
+        <v>54257.120220599987</v>
+      </c>
+      <c r="F6" s="10">
+        <v>3.1222927114860181E-2</v>
+      </c>
+      <c r="G6" s="10">
+        <v>4.4066793598312361E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1104497.8864203531</v>
+      </c>
+      <c r="E7" s="3">
+        <v>55926.329561999992</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1.456969533637424E-2</v>
+      </c>
+      <c r="G7" s="10">
+        <v>1.725521704280945E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1083208.9167629869</v>
+      </c>
+      <c r="E8" s="3">
+        <v>110639.49239553</v>
+      </c>
+      <c r="F8" s="10">
+        <v>6.9333248439685724E-3</v>
+      </c>
+      <c r="G8" s="10">
+        <v>1.1143475296256969E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1077864.821598877</v>
+      </c>
+      <c r="E9" s="3">
+        <v>73997.227386940009</v>
+      </c>
+      <c r="F9" s="10">
+        <v>9.7692142174449353E-3</v>
+      </c>
+      <c r="G9" s="10">
+        <v>9.558347653642385E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D10" s="3">
+        <v>729412.67096789309</v>
+      </c>
+      <c r="E10" s="3">
+        <v>60313.34351775</v>
+      </c>
+      <c r="F10" s="10">
+        <v>3.7694938920620688E-4</v>
+      </c>
+      <c r="G10" s="10">
+        <v>1.654533485954597E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D11" s="3">
+        <v>648447.24948227091</v>
+      </c>
+      <c r="E11" s="3">
+        <v>22130.276711350001</v>
+      </c>
+      <c r="F11" s="10">
+        <v>1.068848483528837E-2</v>
+      </c>
+      <c r="G11" s="10">
+        <v>8.5913209572516789E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D12" s="3">
+        <v>647963.01508706179</v>
+      </c>
+      <c r="E12" s="3">
+        <v>30679.58334573</v>
+      </c>
+      <c r="F12" s="10">
+        <v>6.9744795028248326E-4</v>
+      </c>
+      <c r="G12" s="10">
+        <v>1.104087647419581E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D13" s="3">
+        <v>585416.38894337451</v>
+      </c>
+      <c r="E13" s="3">
+        <v>80201.013479729998</v>
+      </c>
+      <c r="F13" s="10">
+        <v>3.0546519921711193E-4</v>
+      </c>
+      <c r="G13" s="10">
+        <v>1.7612261076438901E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="3">
+        <f>MEDIAN(D2:D13)</f>
+        <v>1093853.40159167</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3">
+        <f>AVERAGE(D2:D7)</f>
+        <v>1598973.9542343842</v>
+      </c>
+      <c r="E17" s="3">
+        <f t="shared" ref="E17:G17" si="0">AVERAGE(E2:E7)</f>
+        <v>58752.201807741658</v>
+      </c>
+      <c r="F17" s="4">
+        <f t="shared" si="0"/>
+        <v>1.2079395573083082E-2</v>
+      </c>
+      <c r="G17" s="4">
+        <f t="shared" si="0"/>
+        <v>2.5947743971152693E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="3">
+        <f>AVERAGE(D8:D13)</f>
+        <v>795385.51047374401</v>
+      </c>
+      <c r="E18" s="3">
+        <f t="shared" ref="E18:G18" si="1">AVERAGE(E8:E13)</f>
+        <v>62993.48947283833</v>
+      </c>
+      <c r="F18" s="4">
+        <f t="shared" si="1"/>
+        <v>4.7951477392346132E-3</v>
+      </c>
+      <c r="G18" s="4">
+        <f t="shared" si="1"/>
+        <v>2.2454820234090326E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="3">
+        <f>D17/D18</f>
+        <v>2.0103131540352179</v>
+      </c>
+      <c r="E20" s="3">
+        <f t="shared" ref="E20:G20" si="2">E17/E18</f>
+        <v>0.93267101567812905</v>
+      </c>
+      <c r="F20" s="3">
+        <f t="shared" si="2"/>
+        <v>2.5190872586151345</v>
+      </c>
+      <c r="G20" s="3">
+        <f t="shared" si="2"/>
+        <v>1.1555534045986038</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D2:D13">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E13">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F13">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G13">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17:D18">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E18">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17:F18">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G18">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="93" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D2" s="3">
+        <v>9937990.5894197039</v>
+      </c>
+      <c r="E2" s="3">
+        <v>137654.50809200999</v>
+      </c>
+      <c r="F2" s="4">
+        <v>2.451646095414645E-3</v>
+      </c>
+      <c r="G2" s="4">
+        <v>7.6188786690442915E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D3" s="3">
+        <v>9153211.3096406423</v>
+      </c>
+      <c r="E3" s="3">
+        <v>158802.14720132999</v>
+      </c>
+      <c r="F3" s="4">
+        <v>2.8137256066412789E-3</v>
+      </c>
+      <c r="G3" s="4">
+        <v>2.4032687441319662E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D4" s="3">
+        <v>8323850.3002414759</v>
+      </c>
+      <c r="E4" s="3">
+        <v>69747.682037220002</v>
+      </c>
+      <c r="F4" s="4">
+        <v>3.3950559124479012E-3</v>
+      </c>
+      <c r="G4" s="4">
+        <v>9.6936097165093425E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D5" s="3">
+        <v>7695797.0900557945</v>
+      </c>
+      <c r="E5" s="3">
+        <v>86242.724574749998</v>
+      </c>
+      <c r="F5" s="4">
+        <v>2.8921735657111581E-3</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1.1051378185227779E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D6" s="3">
+        <v>5034263.5495518269</v>
+      </c>
+      <c r="E6" s="3">
+        <v>65873.429441999993</v>
+      </c>
+      <c r="F6" s="4">
+        <v>2.9423350149191101E-3</v>
+      </c>
+      <c r="G6" s="4">
+        <v>3.4897071466789652E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D7" s="3">
+        <v>4961117.4365704898</v>
+      </c>
+      <c r="E7" s="3">
+        <v>63209.692581750001</v>
+      </c>
+      <c r="F7" s="4">
+        <v>4.351387458407175E-3</v>
+      </c>
+      <c r="G7" s="4">
+        <v>5.6592795928781631E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D8" s="3">
+        <v>4783385.1798815951</v>
+      </c>
+      <c r="E8" s="3">
+        <v>64669.840333150009</v>
+      </c>
+      <c r="F8" s="4">
+        <v>2.0954023999737231E-3</v>
+      </c>
+      <c r="G8" s="4">
+        <v>5.9056880507593645E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D9" s="3">
+        <v>4448196.0441567702</v>
+      </c>
+      <c r="E9" s="3">
+        <v>96473.926682400008</v>
+      </c>
+      <c r="F9" s="4">
+        <v>4.425446074207404E-4</v>
+      </c>
+      <c r="G9" s="4">
+        <v>2.154034060250509E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1252686.154182706</v>
+      </c>
+      <c r="E10" s="3">
+        <v>9796.3168782600005</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0.13430184443805829</v>
+      </c>
+      <c r="G10" s="4">
+        <v>5.218380319387952E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1194490.274669243</v>
+      </c>
+      <c r="E11" s="3">
+        <v>19231.118310289999</v>
+      </c>
+      <c r="F11" s="4">
+        <v>5.2147019888250969E-3</v>
+      </c>
+      <c r="G11" s="4">
+        <v>4.9058279907476332E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1165717.934645507</v>
+      </c>
+      <c r="E12" s="3">
+        <v>8785.8682089999984</v>
+      </c>
+      <c r="F12" s="4">
+        <v>1.025148686019859E-2</v>
+      </c>
+      <c r="G12" s="4">
+        <v>1.7444704536200269E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1063712.5319653209</v>
+      </c>
+      <c r="E13" s="3">
+        <v>8180.2586681400007</v>
+      </c>
+      <c r="F13" s="4">
+        <v>1.6866644248961379E-2</v>
+      </c>
+      <c r="G13" s="4">
+        <v>6.3103132179727491E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="3">
+        <f>MEDIAN(D2:D13)</f>
+        <v>4872251.3082260424</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3">
+        <f>AVERAGE(D2:D7)</f>
+        <v>7517705.0459133228</v>
+      </c>
+      <c r="E17" s="3">
+        <f t="shared" ref="E17:G17" si="0">AVERAGE(E2:E7)</f>
+        <v>96921.697321510001</v>
+      </c>
+      <c r="F17" s="4">
+        <f t="shared" si="0"/>
+        <v>3.141053942256878E-3</v>
+      </c>
+      <c r="G17" s="4">
+        <f t="shared" si="0"/>
+        <v>1.0257590125276369E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="3">
+        <f>AVERAGE(D8:D13)</f>
+        <v>2318031.3532501906</v>
+      </c>
+      <c r="E18" s="3">
+        <f t="shared" ref="E18:G18" si="1">AVERAGE(E8:E13)</f>
+        <v>34522.888180206675</v>
+      </c>
+      <c r="F18" s="4">
+        <f t="shared" si="1"/>
+        <v>2.8195437423906299E-2</v>
+      </c>
+      <c r="G18" s="4">
+        <f t="shared" si="1"/>
+        <v>4.3731190154563726E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D23" s="3">
+        <v>5034263.5495518269</v>
+      </c>
+      <c r="E23" s="3">
+        <v>65873.429441999993</v>
+      </c>
+      <c r="F23" s="4">
+        <v>2.9423350149191101E-3</v>
+      </c>
+      <c r="G23" s="4">
+        <v>3.4897071466789652E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D24" s="3">
+        <v>4961117.4365704898</v>
+      </c>
+      <c r="E24" s="3">
+        <v>63209.692581750001</v>
+      </c>
+      <c r="F24" s="4">
+        <v>4.351387458407175E-3</v>
+      </c>
+      <c r="G24" s="4">
+        <v>5.6592795928781631E-4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D25" s="3">
+        <v>4783385.1798815951</v>
+      </c>
+      <c r="E25" s="3">
+        <v>64669.840333150009</v>
+      </c>
+      <c r="F25" s="4">
+        <v>2.0954023999737231E-3</v>
+      </c>
+      <c r="G25" s="4">
+        <v>5.9056880507593645E-4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D26" s="3">
+        <v>4448196.0441567702</v>
+      </c>
+      <c r="E26" s="3">
+        <v>96473.926682400008</v>
+      </c>
+      <c r="F26" s="4">
+        <v>4.425446074207404E-4</v>
+      </c>
+      <c r="G26" s="4">
+        <v>2.154034060250509E-4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="3">
+        <f>AVERAGE(D23:D24)</f>
+        <v>4997690.4930611588</v>
+      </c>
+      <c r="E28" s="3">
+        <f t="shared" ref="E28:G28" si="2">AVERAGE(E23:E24)</f>
+        <v>64541.561011874997</v>
+      </c>
+      <c r="F28" s="4">
+        <f t="shared" si="2"/>
+        <v>3.6468612366631426E-3</v>
+      </c>
+      <c r="G28" s="4">
+        <f t="shared" si="2"/>
+        <v>4.5744933697785639E-4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="3">
+        <f>AVERAGE(D25:D26)</f>
+        <v>4615790.6120191831</v>
+      </c>
+      <c r="E29" s="3">
+        <f t="shared" ref="E29:G29" si="3">AVERAGE(E25:E26)</f>
+        <v>80571.883507775012</v>
+      </c>
+      <c r="F29" s="4">
+        <f t="shared" si="3"/>
+        <v>1.2689735036972318E-3</v>
+      </c>
+      <c r="G29" s="4">
+        <f t="shared" si="3"/>
+        <v>4.0298610555049367E-4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" s="3">
+        <f>D28/D29</f>
+        <v>1.0827376961267559</v>
+      </c>
+      <c r="E31" s="3">
+        <f t="shared" ref="E31:G31" si="4">E28/E29</f>
+        <v>0.80104322006630113</v>
+      </c>
+      <c r="F31" s="3">
+        <f t="shared" si="4"/>
+        <v>2.8738671264906555</v>
+      </c>
+      <c r="G31" s="3">
+        <f t="shared" si="4"/>
+        <v>1.1351491544676557</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D2:D13">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E13">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F13">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G13">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17:D18">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E18">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17:F18">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G18">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D23:D26">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23:E26">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F23:F26">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23:G26">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D28:D29">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28:E29">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F28:F29">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28:G29">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -3647,6 +4026,1205 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="97.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D2" s="3">
+        <v>3292837.3871137551</v>
+      </c>
+      <c r="E2" s="3">
+        <v>5258.5701260400001</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1.0604360748915839E-2</v>
+      </c>
+      <c r="G2" s="4">
+        <v>1.868819729404374E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D3" s="3">
+        <v>3097084.3107878752</v>
+      </c>
+      <c r="E3" s="3">
+        <v>4162.4721680000002</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1.4081114307645259E-3</v>
+      </c>
+      <c r="G3" s="4">
+        <v>3.9573959548935052E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2652658.7944572391</v>
+      </c>
+      <c r="E4" s="3">
+        <v>4253.6615775199998</v>
+      </c>
+      <c r="F4" s="4">
+        <v>2.8806641846538372E-3</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1.8380008135386839E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2480166.278394436</v>
+      </c>
+      <c r="E5" s="3">
+        <v>4510.0316159999993</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1.003512255644462E-3</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1.2206708220113729E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D6" s="3">
+        <v>331647.0310656284</v>
+      </c>
+      <c r="E6" s="3">
+        <v>964.84556195999994</v>
+      </c>
+      <c r="F6" s="4">
+        <v>7.4163848413873461E-4</v>
+      </c>
+      <c r="G6" s="4">
+        <v>3.6380912535570372E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D7" s="3">
+        <v>255261.79722573471</v>
+      </c>
+      <c r="E7" s="3">
+        <v>888.20773440000005</v>
+      </c>
+      <c r="F7" s="4">
+        <v>1.2066660967819649E-3</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2.863735386990569E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D8" s="3">
+        <v>238996.75153477999</v>
+      </c>
+      <c r="E8" s="3">
+        <v>863.40619829999991</v>
+      </c>
+      <c r="F8" s="4">
+        <v>7.0023981897559661E-4</v>
+      </c>
+      <c r="G8" s="4">
+        <v>9.1753228267274999E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D9" s="3">
+        <v>218314.63160777459</v>
+      </c>
+      <c r="E9" s="3">
+        <v>897.65553599999998</v>
+      </c>
+      <c r="F9" s="4">
+        <v>4.6312642581418888E-4</v>
+      </c>
+      <c r="G9" s="4">
+        <v>5.3328786021100191E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D10" s="3">
+        <v>177476.11420904889</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1454.99992092</v>
+      </c>
+      <c r="F10" s="4">
+        <v>2.7347370558508639E-4</v>
+      </c>
+      <c r="G10" s="4">
+        <v>8.7625687236728058E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D11" s="3">
+        <v>149725.9222474432</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1319.2765561000001</v>
+      </c>
+      <c r="F11" s="4">
+        <v>9.5143491498901212E-3</v>
+      </c>
+      <c r="G11" s="4">
+        <v>8.6555389370039323E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D12" s="3">
+        <v>123407.0292947656</v>
+      </c>
+      <c r="E12" s="3">
+        <v>769.72569599999997</v>
+      </c>
+      <c r="F12" s="4">
+        <v>1.643806367093142E-3</v>
+      </c>
+      <c r="G12" s="4">
+        <v>4.963035559098705E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D13" s="3">
+        <v>118648.02708896549</v>
+      </c>
+      <c r="E13" s="3">
+        <v>640.62859736000007</v>
+      </c>
+      <c r="F13" s="4">
+        <v>4.2703506076277667E-2</v>
+      </c>
+      <c r="G13" s="4">
+        <v>7.645975624855611E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="3">
+        <f>MEDIAN(D2:D13)</f>
+        <v>247129.27438025735</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3">
+        <f>AVERAGE(D2:D7)</f>
+        <v>2018275.9331741116</v>
+      </c>
+      <c r="E17" s="3">
+        <f t="shared" ref="E17:G17" si="0">AVERAGE(E2:E7)</f>
+        <v>3339.6314639866664</v>
+      </c>
+      <c r="F17" s="4">
+        <f t="shared" si="0"/>
+        <v>2.974158866816561E-3</v>
+      </c>
+      <c r="G17" s="4">
+        <f t="shared" si="0"/>
+        <v>2.0187386386990346E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="3">
+        <f>AVERAGE(D8:D13)</f>
+        <v>171094.74599712962</v>
+      </c>
+      <c r="E18" s="3">
+        <f t="shared" ref="E18:G18" si="1">AVERAGE(E8:E13)</f>
+        <v>990.94875077999995</v>
+      </c>
+      <c r="F18" s="4">
+        <f t="shared" si="1"/>
+        <v>9.2164169239392999E-3</v>
+      </c>
+      <c r="G18" s="4">
+        <f t="shared" si="1"/>
+        <v>3.4335388058007936E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="3">
+        <f>D17/D18</f>
+        <v>11.796247286330882</v>
+      </c>
+      <c r="E20" s="3">
+        <f t="shared" ref="E20:G20" si="2">E17/E18</f>
+        <v>3.3701353993917049</v>
+      </c>
+      <c r="F20" s="3">
+        <f t="shared" si="2"/>
+        <v>0.32270229215556578</v>
+      </c>
+      <c r="G20" s="3">
+        <f t="shared" si="2"/>
+        <v>0.58794694129813696</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D24" s="3">
+        <v>3292837.3871137551</v>
+      </c>
+      <c r="E24" s="3">
+        <v>5258.5701260400001</v>
+      </c>
+      <c r="F24" s="4">
+        <v>1.0604360748915839E-2</v>
+      </c>
+      <c r="G24" s="4">
+        <v>1.868819729404374E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D25" s="3">
+        <v>3097084.3107878752</v>
+      </c>
+      <c r="E25" s="3">
+        <v>4162.4721680000002</v>
+      </c>
+      <c r="F25" s="4">
+        <v>1.4081114307645259E-3</v>
+      </c>
+      <c r="G25" s="4">
+        <v>3.9573959548935052E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D26" s="3">
+        <v>2652658.7944572391</v>
+      </c>
+      <c r="E26" s="3">
+        <v>4253.6615775199998</v>
+      </c>
+      <c r="F26" s="4">
+        <v>2.8806641846538372E-3</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1.8380008135386839E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D27" s="3">
+        <v>2480166.278394436</v>
+      </c>
+      <c r="E27" s="3">
+        <v>4510.0316159999993</v>
+      </c>
+      <c r="F27" s="4">
+        <v>1.003512255644462E-3</v>
+      </c>
+      <c r="G27" s="4">
+        <v>1.2206708220113729E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="3">
+        <f>AVERAGE(D24:D25)</f>
+        <v>3194960.8489508154</v>
+      </c>
+      <c r="E29" s="3">
+        <f t="shared" ref="E29:G30" si="3">AVERAGE(E24:E25)</f>
+        <v>4710.5211470200002</v>
+      </c>
+      <c r="F29" s="4">
+        <f t="shared" si="3"/>
+        <v>6.0062360898401829E-3</v>
+      </c>
+      <c r="G29" s="4">
+        <f t="shared" si="3"/>
+        <v>2.9131078421489398E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="3">
+        <f>AVERAGE(D26:D27)</f>
+        <v>2566412.5364258373</v>
+      </c>
+      <c r="E30" s="3">
+        <f t="shared" ref="E30:G30" si="4">AVERAGE(E26:E27)</f>
+        <v>4381.8465967599996</v>
+      </c>
+      <c r="F30" s="4">
+        <f t="shared" si="4"/>
+        <v>1.9420882201491496E-3</v>
+      </c>
+      <c r="G30" s="4">
+        <f t="shared" si="4"/>
+        <v>1.5293358177750284E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="3">
+        <f>D29/D30</f>
+        <v>1.2449132022244318</v>
+      </c>
+      <c r="E32" s="3">
+        <f t="shared" ref="E32:G32" si="5">E29/E30</f>
+        <v>1.0750082283809359</v>
+      </c>
+      <c r="F32" s="3">
+        <f t="shared" si="5"/>
+        <v>3.092669028896593</v>
+      </c>
+      <c r="G32" s="3">
+        <f t="shared" si="5"/>
+        <v>1.9048189470819483</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState ref="A2:G13">
+    <sortCondition descending="1" ref="D2:D13"/>
+  </sortState>
+  <conditionalFormatting sqref="D2:D13">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E13">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F13">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G13">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17:D18">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E18">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17:F18">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G18">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D24:D27">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24:E27">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F24:F27">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G24:G27">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D29:D30">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E29:E30">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F29:F30">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29:G30">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="73" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D2" s="3">
+        <v>971947.1589226143</v>
+      </c>
+      <c r="E2" s="3">
+        <v>21731.663739110001</v>
+      </c>
+      <c r="F2" s="4">
+        <v>3.0282081846115981E-5</v>
+      </c>
+      <c r="G2" s="4">
+        <v>5.0206173563068553E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D3" s="3">
+        <v>950234.48563991196</v>
+      </c>
+      <c r="E3" s="3">
+        <v>3253.0570836699999</v>
+      </c>
+      <c r="F3" s="4">
+        <v>3.2666995157709352E-4</v>
+      </c>
+      <c r="G3" s="4">
+        <v>1.167450820049999E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D4" s="3">
+        <v>840420.70663642394</v>
+      </c>
+      <c r="E4" s="3">
+        <v>22097.462448999999</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1.047846559460851E-5</v>
+      </c>
+      <c r="G4" s="4">
+        <v>8.9257472528899238E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D5" s="3">
+        <v>130071.2900498806</v>
+      </c>
+      <c r="E5" s="3">
+        <v>866.32844524999996</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1.8830176464184379E-3</v>
+      </c>
+      <c r="G5" s="4">
+        <v>2.5735129813919731E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D6" s="3">
+        <v>118956.3612196709</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1090.8420791399999</v>
+      </c>
+      <c r="F6" s="4">
+        <v>6.857037460360029E-4</v>
+      </c>
+      <c r="G6" s="4">
+        <v>4.8025762850386331E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D7" s="3">
+        <v>106346.7598437235</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1736.36278023</v>
+      </c>
+      <c r="F7" s="4">
+        <v>2.7534118528886658E-3</v>
+      </c>
+      <c r="G7" s="4">
+        <v>9.5257384161442811E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D8" s="3">
+        <v>85809.083743767143</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2740.6294030899999</v>
+      </c>
+      <c r="F8" s="4">
+        <v>3.444045779906578E-2</v>
+      </c>
+      <c r="G8" s="4">
+        <v>2.7573625574766692E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="3">
+        <f>MEDIAN(D2:D8)</f>
+        <v>130071.2900498806</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="6"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="3">
+        <f>AVERAGE(D2:D4)</f>
+        <v>920867.45039964991</v>
+      </c>
+      <c r="E12" s="3">
+        <f t="shared" ref="E12:G12" si="0">AVERAGE(E2:E4)</f>
+        <v>15694.061090593334</v>
+      </c>
+      <c r="F12" s="4">
+        <f t="shared" si="0"/>
+        <v>1.2247683300593934E-4</v>
+      </c>
+      <c r="G12" s="4">
+        <f t="shared" si="0"/>
+        <v>5.0379384764155924E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="3">
+        <f>AVERAGE(D6:D8)</f>
+        <v>103704.06826905387</v>
+      </c>
+      <c r="E13" s="3">
+        <f t="shared" ref="E13:G13" si="1">AVERAGE(E6:E8)</f>
+        <v>1855.9447541533334</v>
+      </c>
+      <c r="F13" s="4">
+        <f t="shared" si="1"/>
+        <v>1.2626524465996816E-2</v>
+      </c>
+      <c r="G13" s="4">
+        <f t="shared" si="1"/>
+        <v>3.4272441001319369E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="3">
+        <f>D12/D13</f>
+        <v>8.8797620553372667</v>
+      </c>
+      <c r="E15" s="3">
+        <f t="shared" ref="E15:G15" si="2">E12/E13</f>
+        <v>8.4561035857734002</v>
+      </c>
+      <c r="F15" s="3">
+        <f t="shared" si="2"/>
+        <v>9.6999640190591641E-3</v>
+      </c>
+      <c r="G15" s="3">
+        <f t="shared" si="2"/>
+        <v>1.469967801891219</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D2:D8">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E8">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F8">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G8">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12:D13">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12:E13">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F12:F13">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G12:G13">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D19:D22">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19:E22">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F19:F22">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19:G22">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3681,10 +5259,10 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="8" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3710,10 +5288,10 @@
       <c r="G2" s="4">
         <v>9.1204876912707078E-4</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="8" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3739,10 +5317,10 @@
       <c r="G3" s="4">
         <v>1.009990774998547E-3</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="8" t="s">
         <v>68</v>
       </c>
     </row>
@@ -3791,7 +5369,7 @@
       <c r="G5" s="4">
         <v>6.8807976565944413E-4</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="9" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4075,7 +5653,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D19">
@@ -4084,10 +5662,10 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C20" s="7"/>
+      <c r="C20" s="6"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C21" s="7"/>
+      <c r="C21" s="6"/>
       <c r="D21" s="1" t="s">
         <v>63</v>
       </c>
@@ -4102,7 +5680,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>79</v>
       </c>
       <c r="D22" s="2">
@@ -4123,7 +5701,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="6" t="s">
         <v>80</v>
       </c>
       <c r="D23" s="2">
@@ -4193,7 +5771,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D22:D23">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4205,7 +5783,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E22:E23">
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4217,7 +5795,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F22:F23">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4229,7 +5807,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G22:G23">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4243,951 +5821,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="93" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C2" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D2" s="3">
-        <v>9937990.5894197039</v>
-      </c>
-      <c r="E2" s="3">
-        <v>137654.50809200999</v>
-      </c>
-      <c r="F2" s="4">
-        <v>2.451646095414645E-3</v>
-      </c>
-      <c r="G2" s="4">
-        <v>7.6188786690442915E-4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D3" s="3">
-        <v>9153211.3096406423</v>
-      </c>
-      <c r="E3" s="3">
-        <v>158802.14720132999</v>
-      </c>
-      <c r="F3" s="4">
-        <v>2.8137256066412789E-3</v>
-      </c>
-      <c r="G3" s="4">
-        <v>2.4032687441319662E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C4" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D4" s="3">
-        <v>8323850.3002414759</v>
-      </c>
-      <c r="E4" s="3">
-        <v>69747.682037220002</v>
-      </c>
-      <c r="F4" s="4">
-        <v>3.3950559124479012E-3</v>
-      </c>
-      <c r="G4" s="4">
-        <v>9.6936097165093425E-4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D5" s="3">
-        <v>7695797.0900557945</v>
-      </c>
-      <c r="E5" s="3">
-        <v>86242.724574749998</v>
-      </c>
-      <c r="F5" s="4">
-        <v>2.8921735657111581E-3</v>
-      </c>
-      <c r="G5" s="4">
-        <v>1.1051378185227779E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D6" s="3">
-        <v>5034263.5495518269</v>
-      </c>
-      <c r="E6" s="3">
-        <v>65873.429441999993</v>
-      </c>
-      <c r="F6" s="4">
-        <v>2.9423350149191101E-3</v>
-      </c>
-      <c r="G6" s="4">
-        <v>3.4897071466789652E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D7" s="3">
-        <v>4961117.4365704898</v>
-      </c>
-      <c r="E7" s="3">
-        <v>63209.692581750001</v>
-      </c>
-      <c r="F7" s="4">
-        <v>4.351387458407175E-3</v>
-      </c>
-      <c r="G7" s="4">
-        <v>5.6592795928781631E-4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D8" s="3">
-        <v>4783385.1798815951</v>
-      </c>
-      <c r="E8" s="3">
-        <v>64669.840333150009</v>
-      </c>
-      <c r="F8" s="4">
-        <v>2.0954023999737231E-3</v>
-      </c>
-      <c r="G8" s="4">
-        <v>5.9056880507593645E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C9" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D9" s="3">
-        <v>4448196.0441567702</v>
-      </c>
-      <c r="E9" s="3">
-        <v>96473.926682400008</v>
-      </c>
-      <c r="F9" s="4">
-        <v>4.425446074207404E-4</v>
-      </c>
-      <c r="G9" s="4">
-        <v>2.154034060250509E-4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D10" s="3">
-        <v>1252686.154182706</v>
-      </c>
-      <c r="E10" s="3">
-        <v>9796.3168782600005</v>
-      </c>
-      <c r="F10" s="4">
-        <v>0.13430184443805829</v>
-      </c>
-      <c r="G10" s="4">
-        <v>5.218380319387952E-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D11" s="3">
-        <v>1194490.274669243</v>
-      </c>
-      <c r="E11" s="3">
-        <v>19231.118310289999</v>
-      </c>
-      <c r="F11" s="4">
-        <v>5.2147019888250969E-3</v>
-      </c>
-      <c r="G11" s="4">
-        <v>4.9058279907476332E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C12" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D12" s="3">
-        <v>1165717.934645507</v>
-      </c>
-      <c r="E12" s="3">
-        <v>8785.8682089999984</v>
-      </c>
-      <c r="F12" s="4">
-        <v>1.025148686019859E-2</v>
-      </c>
-      <c r="G12" s="4">
-        <v>1.7444704536200269E-4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D13" s="3">
-        <v>1063712.5319653209</v>
-      </c>
-      <c r="E13" s="3">
-        <v>8180.2586681400007</v>
-      </c>
-      <c r="F13" s="4">
-        <v>1.6866644248961379E-2</v>
-      </c>
-      <c r="G13" s="4">
-        <v>6.3103132179727491E-4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="3">
-        <f>MEDIAN(D2:D13)</f>
-        <v>4872251.3082260424</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="3">
-        <f>AVERAGE(D2:D7)</f>
-        <v>7517705.0459133228</v>
-      </c>
-      <c r="E17" s="3">
-        <f t="shared" ref="E17:G17" si="0">AVERAGE(E2:E7)</f>
-        <v>96921.697321510001</v>
-      </c>
-      <c r="F17" s="4">
-        <f t="shared" si="0"/>
-        <v>3.141053942256878E-3</v>
-      </c>
-      <c r="G17" s="4">
-        <f t="shared" si="0"/>
-        <v>1.0257590125276369E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="3">
-        <f>AVERAGE(D8:D13)</f>
-        <v>2318031.3532501906</v>
-      </c>
-      <c r="E18" s="3">
-        <f t="shared" ref="E18:G18" si="1">AVERAGE(E8:E13)</f>
-        <v>34522.888180206675</v>
-      </c>
-      <c r="F18" s="4">
-        <f t="shared" si="1"/>
-        <v>2.8195437423906299E-2</v>
-      </c>
-      <c r="G18" s="4">
-        <f t="shared" si="1"/>
-        <v>4.3731190154563726E-4</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="D2:D13">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E13">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F13">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G13">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17:D18">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E18">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F17:F18">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G18">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="120.28515625" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D2" s="3">
-        <v>2312764.5271400302</v>
-      </c>
-      <c r="E2" s="3">
-        <v>35420.059524999997</v>
-      </c>
-      <c r="F2" s="11">
-        <v>5.6205038026400662E-3</v>
-      </c>
-      <c r="G2" s="11">
-        <v>1.8864917830766969E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D3" s="3">
-        <v>2056038.0691327541</v>
-      </c>
-      <c r="E3" s="3">
-        <v>35306.169047820003</v>
-      </c>
-      <c r="F3" s="11">
-        <v>7.4585983781851224E-3</v>
-      </c>
-      <c r="G3" s="11">
-        <v>1.5495337612500891E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D4" s="3">
-        <v>1713109.9518803279</v>
-      </c>
-      <c r="E4" s="3">
-        <v>77023.192478700003</v>
-      </c>
-      <c r="F4" s="11">
-        <v>9.4864560705148846E-3</v>
-      </c>
-      <c r="G4" s="11">
-        <v>3.0572532777723999E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D5" s="3">
-        <v>1230284.2821290109</v>
-      </c>
-      <c r="E5" s="3">
-        <v>94580.340012330009</v>
-      </c>
-      <c r="F5" s="11">
-        <v>4.1181927359240046E-3</v>
-      </c>
-      <c r="G5" s="11">
-        <v>2.9431664964802489E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C6" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D6" s="3">
-        <v>1177149.00870383</v>
-      </c>
-      <c r="E6" s="3">
-        <v>54257.120220599987</v>
-      </c>
-      <c r="F6" s="11">
-        <v>3.1222927114860181E-2</v>
-      </c>
-      <c r="G6" s="11">
-        <v>4.4066793598312361E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D7" s="3">
-        <v>1104497.8864203531</v>
-      </c>
-      <c r="E7" s="3">
-        <v>55926.329561999992</v>
-      </c>
-      <c r="F7" s="11">
-        <v>1.456969533637424E-2</v>
-      </c>
-      <c r="G7" s="11">
-        <v>1.725521704280945E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D8" s="3">
-        <v>1083208.9167629869</v>
-      </c>
-      <c r="E8" s="3">
-        <v>110639.49239553</v>
-      </c>
-      <c r="F8" s="11">
-        <v>6.9333248439685724E-3</v>
-      </c>
-      <c r="G8" s="11">
-        <v>1.1143475296256969E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D9" s="3">
-        <v>1077864.821598877</v>
-      </c>
-      <c r="E9" s="3">
-        <v>73997.227386940009</v>
-      </c>
-      <c r="F9" s="11">
-        <v>9.7692142174449353E-3</v>
-      </c>
-      <c r="G9" s="11">
-        <v>9.558347653642385E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D10" s="3">
-        <v>729412.67096789309</v>
-      </c>
-      <c r="E10" s="3">
-        <v>60313.34351775</v>
-      </c>
-      <c r="F10" s="11">
-        <v>3.7694938920620688E-4</v>
-      </c>
-      <c r="G10" s="11">
-        <v>1.654533485954597E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D11" s="3">
-        <v>648447.24948227091</v>
-      </c>
-      <c r="E11" s="3">
-        <v>22130.276711350001</v>
-      </c>
-      <c r="F11" s="11">
-        <v>1.068848483528837E-2</v>
-      </c>
-      <c r="G11" s="11">
-        <v>8.5913209572516789E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C12" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D12" s="3">
-        <v>647963.01508706179</v>
-      </c>
-      <c r="E12" s="3">
-        <v>30679.58334573</v>
-      </c>
-      <c r="F12" s="11">
-        <v>6.9744795028248326E-4</v>
-      </c>
-      <c r="G12" s="11">
-        <v>1.104087647419581E-4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C13" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D13" s="3">
-        <v>585416.38894337451</v>
-      </c>
-      <c r="E13" s="3">
-        <v>80201.013479729998</v>
-      </c>
-      <c r="F13" s="11">
-        <v>3.0546519921711193E-4</v>
-      </c>
-      <c r="G13" s="11">
-        <v>1.7612261076438901E-4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="3">
-        <f>MEDIAN(D2:D13)</f>
-        <v>1093853.40159167</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="3">
-        <f>AVERAGE(D2:D7)</f>
-        <v>1598973.9542343842</v>
-      </c>
-      <c r="E17" s="3">
-        <f t="shared" ref="E17:G17" si="0">AVERAGE(E2:E7)</f>
-        <v>58752.201807741658</v>
-      </c>
-      <c r="F17" s="4">
-        <f t="shared" si="0"/>
-        <v>1.2079395573083082E-2</v>
-      </c>
-      <c r="G17" s="4">
-        <f t="shared" si="0"/>
-        <v>2.5947743971152693E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="3">
-        <f>AVERAGE(D8:D13)</f>
-        <v>795385.51047374401</v>
-      </c>
-      <c r="E18" s="3">
-        <f t="shared" ref="E18:G18" si="1">AVERAGE(E8:E13)</f>
-        <v>62993.48947283833</v>
-      </c>
-      <c r="F18" s="4">
-        <f t="shared" si="1"/>
-        <v>4.7951477392346132E-3</v>
-      </c>
-      <c r="G18" s="4">
-        <f t="shared" si="1"/>
-        <v>2.2454820234090326E-3</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="3">
-        <f>D17/D18</f>
-        <v>2.0103131540352179</v>
-      </c>
-      <c r="E20" s="3">
-        <f t="shared" ref="E20:G20" si="2">E17/E18</f>
-        <v>0.93267101567812905</v>
-      </c>
-      <c r="F20" s="3">
-        <f t="shared" si="2"/>
-        <v>2.5190872586151345</v>
-      </c>
-      <c r="G20" s="3">
-        <f t="shared" si="2"/>
-        <v>1.1555534045986038</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="D2:D13">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E13">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F13">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G13">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17:D18">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E18">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F17:F18">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G18">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>